<commit_message>
no such element Test 11
</commit_message>
<xml_diff>
--- a/src/test/resources/login.xlsx
+++ b/src/test/resources/login.xlsx
@@ -27,12 +27,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="25">
   <si>
     <t>Email</t>
   </si>
   <si>
-    <t>Mật khẩu</t>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Test Case</t>
   </si>
   <si>
     <t>innologic25.team@gmail.com</t>
@@ -41,10 +44,64 @@
     <t>innologic2025</t>
   </si>
   <si>
-    <t>testuser01@example.com</t>
-  </si>
-  <si>
-    <t>test@1234</t>
+    <t>testSuccess</t>
+  </si>
+  <si>
+    <t>invalid_email@gmail.com</t>
+  </si>
+  <si>
+    <t>testNonExistentEmail</t>
+  </si>
+  <si>
+    <t>invalid-email-format</t>
+  </si>
+  <si>
+    <t>testInvalidEmailFormat</t>
+  </si>
+  <si>
+    <t>testEmptyPassword</t>
+  </si>
+  <si>
+    <t>testEmptyEmail</t>
+  </si>
+  <si>
+    <t>testEmptyEmailAndPassword</t>
+  </si>
+  <si>
+    <t>user!@gmail.com</t>
+  </si>
+  <si>
+    <t>validPassword123</t>
+  </si>
+  <si>
+    <t>testInvalidEmailSpecialChars</t>
+  </si>
+  <si>
+    <t>user@gmail.com</t>
+  </si>
+  <si>
+    <t>testShortPassword</t>
+  </si>
+  <si>
+    <t>user @gmail.com</t>
+  </si>
+  <si>
+    <t>testEmailContainingSpaces</t>
+  </si>
+  <si>
+    <t>123 456</t>
+  </si>
+  <si>
+    <t>testPasswordContainingSpaces</t>
+  </si>
+  <si>
+    <t>abc</t>
+  </si>
+  <si>
+    <t>abc123</t>
+  </si>
+  <si>
+    <t>testPasswordVisibilityToggle</t>
   </si>
 </sst>
 </file>
@@ -668,12 +725,18 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1208,38 +1271,158 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="1"/>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="33.1111111111111" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="2" max="2" width="25.7777777777778" customWidth="1"/>
+    <col min="3" max="3" width="29.1111111111111" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1"/>
     </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
+    <row r="2" spans="1:4">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="2"/>
     </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
+    <row r="3" spans="1:4">
+      <c r="A3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
+      <c r="C3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="2"/>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="2"/>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="2"/>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="2"/>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="2"/>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="3">
+        <v>12345</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="2"/>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="2"/>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" s="2"/>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="2"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" display="invalid_email@gmail.com" tooltip="mailto:invalid_email@gmail.com"/>
+    <hyperlink ref="A5" r:id="rId2" display="innologic25.team@gmail.com" tooltip="mailto:innologic25.team@gmail.com"/>
+    <hyperlink ref="A9" r:id="rId3" display="user@gmail.com" tooltip="mailto:user@gmail.com"/>
+    <hyperlink ref="A11" r:id="rId3" display="user@gmail.com" tooltip="mailto:user@gmail.com"/>
+    <hyperlink ref="A2" r:id="rId2" display="innologic25.team@gmail.com" tooltip="mailto:innologic25.team@gmail.com"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>

</xml_diff>